<commit_message>
Restore working state of 'dati' folder: fix 1_estrai_ddt_consegne.py regression and include new 'crea_distinta_magazzino.py' script
</commit_message>
<xml_diff>
--- a/dati/rientri_ddt.xlsx
+++ b/dati/rientri_ddt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Il mio Drive\AppLogSolution\dati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65BB1855-5025-4F51-B827-2F52C007050D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D660E22D-97DE-4C58-9AF6-05E82227F581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
   <si>
     <t>Codice consegna</t>
   </si>
@@ -86,6 +86,9 @@
   </si>
   <si>
     <t>p2023</t>
+  </si>
+  <si>
+    <t>Allegato con DDT (19/03/2026)</t>
   </si>
 </sst>
 </file>
@@ -426,13 +429,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="20.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="13.36328125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -443,7 +446,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -454,7 +457,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -465,7 +468,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -476,7 +479,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -487,7 +490,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -498,7 +501,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -509,7 +512,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -520,7 +523,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -531,7 +534,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -542,7 +545,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -553,23 +556,29 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>16</v>
       </c>
       <c r="B12" s="1">
         <v>46093</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>17</v>
       </c>
       <c r="B13" s="1">
         <v>46093</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -580,7 +589,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -591,7 +600,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -599,7 +608,7 @@
         <v>46097</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -607,12 +616,15 @@
         <v>46097</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>21</v>
       </c>
       <c r="B18" s="1">
         <v>46093</v>
+      </c>
+      <c r="D18" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Unificazione dati consegne e raffinamento dropdown inserimento
</commit_message>
<xml_diff>
--- a/dati/rientri_ddt.xlsx
+++ b/dati/rientri_ddt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Il mio Drive\AppLogSolution\dati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D660E22D-97DE-4C58-9AF6-05E82227F581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7071F3BD-5D4A-4DE6-9833-8CF5A3F904A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="25">
   <si>
     <t>Codice consegna</t>
   </si>
@@ -89,6 +89,12 @@
   </si>
   <si>
     <t>Allegato con DDT (19/03/2026)</t>
+  </si>
+  <si>
+    <t>p2359</t>
+  </si>
+  <si>
+    <t>p1874</t>
   </si>
 </sst>
 </file>
@@ -429,13 +435,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="20.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="13.36328125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -446,7 +452,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -457,7 +463,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -468,7 +474,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -479,7 +485,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -490,7 +496,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -501,7 +507,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -512,7 +518,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -523,7 +529,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -534,7 +540,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -545,7 +551,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -556,29 +562,29 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>16</v>
       </c>
       <c r="B12" s="1">
         <v>46093</v>
       </c>
-      <c r="D12" t="s">
+      <c r="C12" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>17</v>
       </c>
       <c r="B13" s="1">
         <v>46093</v>
       </c>
-      <c r="D13" t="s">
+      <c r="C13" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -589,7 +595,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -600,31 +606,53 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>19</v>
       </c>
       <c r="B16" s="1">
         <v>46097</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C16" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>20</v>
       </c>
       <c r="B17" s="1">
         <v>46097</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>21</v>
       </c>
       <c r="B18" s="1">
         <v>46093</v>
       </c>
-      <c r="D18" t="s">
+      <c r="C18" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="1">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="1">
+        <v>46100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[v1.34] Fix Inizio Viaggio e tracker GPS 90s
</commit_message>
<xml_diff>
--- a/dati/rientri_ddt.xlsx
+++ b/dati/rientri_ddt.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Il mio Drive\AppLogSolution\dati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AA9BE23-C199-4849-8278-CA2ACDEC64C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42500EAC-F9D3-405C-B8F8-E161058D3536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38070" yWindow="40" windowWidth="12010" windowHeight="13630" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rientri" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="64">
   <si>
     <t>Codice consegna</t>
   </si>
@@ -561,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultColWidth="20.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="13.36328125" style="1" customWidth="1"/>
@@ -1096,6 +1096,62 @@
         <v>63</v>
       </c>
     </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>49</v>
+      </c>
+      <c r="B49" s="1">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>36</v>
+      </c>
+      <c r="B50" s="1">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>50</v>
+      </c>
+      <c r="B51" s="1">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>40</v>
+      </c>
+      <c r="B52" s="1">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>40</v>
+      </c>
+      <c r="B53" s="1">
+        <v>46099</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>51</v>
+      </c>
+      <c r="B54" s="1">
+        <v>46106</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>38</v>
+      </c>
+      <c r="B55" s="1">
+        <v>46106</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>